<commit_message>
docs: expand 12 Wuhan agent knowledge packs and raise every QA library above 50
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/submission/knowledge/A01-武汉总控导游/武汉总控导游QA导入表.xlsx
+++ b/submission/knowledge/A01-武汉总控导游/武汉总控导游QA导入表.xlsx
@@ -877,6 +877,346 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">武大樱花和东湖樱园是一回事吗？</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不是。武大是校园预约；东湖樱花园常单独售票。黄鹤楼又是另一套票。细排请行程规划师，预约请商户助手。</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">辛亥革命纪念馆要预约吗？</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请武汉景点讲解员按博物院须知讲。个人一般免网上预约，南北区闭馆日不同，不要和省博搞混。</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">晴川阁免费吗？</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">日场以晴川阁官网须知为准，常见免费开放；夜游常另计。怎么进请讲解员或商户助手。</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">周一下雨去哪？</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">先远离江边，应急助手管安全。周一省博、古琴台、晴川阁、辛亥南区常闭，改线请行程规划师。</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">老人坐轮椅能上黄鹤楼吗？</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">蛇山有台阶，量力。具体设施问讲解员现场。无障碍细节也可问商户助手。我保证不了每座园都能通轮椅。</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">护照丢了找你？</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">先110，请武汉应急助手。我不代办证件。</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">地铁怎么扫码？</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请武汉交通住宿管家讲乘车码和单程票。我不管实时余票。</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">想买周黑鸭？</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">食品伴手礼请武汉美食顾问。文创请新消费导购。</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">夜游晴川阁等于灯光秀吗？</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不是。灯光秀多在江滩免费看江。夜游晴川阁、夜上黄鹤楼、游船都是另票。请活动预约官拆开讲。</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">带宠物去黄鹤楼？</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">多数文物园限制。请商户助手查公园公众号，不要默认可以带。</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">省博和红楼是一个馆吗？</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不是。省博要官方预约、周一常闭；辛亥革命博物院个人一般免网上预约，南北区闭馆日不同。请讲解员拆开讲。</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">编钟乐舞在黄鹤楼看吗？</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">在湖北省博物馆，须先预约入馆再另购演出票。场次请活动预约官。</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">帮我找黄牛进武大。</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不能。赏樱走学校官方预约。没有名额改东湖听涛或江滩。购票入口请商户助手。</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">被卖假票了。</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">先保证人安全，请应急助手。投诉走12345，不要打已取消的12301。</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">园博园和中山舰今天能和黄鹤楼一起吗？</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">那是跨区点，半天武昌塞不下。请行程规划师按一整天或另日排。</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">吉庆街和户部巷一样吗？</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不是同一条街。过早细节请美食顾问。</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">地铁末班能赶上夜游船吗？</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请交通住宿管家按当晚班次讲，我不报死时刻。活动结束时间问预约官。</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">想买汉绣，怕假。</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">文创认准正规渠道，请新消费导购。工艺讲解请非遗文化官。不给代购微信号。</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">小孩走丢了还先问黄鹤楼吗？</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">先应急助手，原地或服务台，必要时110。景点讲解往后放。</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">热干面芝麻酱过敏。</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">请美食顾问按忌口讲。我不编替代食谱，现场仍要问店员。</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">赏樱与馆</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>